<commit_message>
query deistv contr and excel sum_pr
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -866,34 +866,34 @@
         <v>27.84</v>
       </c>
       <c r="J6" s="11" t="n">
-        <v>1161.44</v>
+        <v>1247.04</v>
       </c>
       <c r="K6" s="11" t="n">
-        <v>1963.19</v>
+        <v>2048.79</v>
       </c>
       <c r="L6" s="11" t="n">
-        <v>2067.59</v>
+        <v>2238.79</v>
       </c>
       <c r="M6" s="11" t="n">
-        <v>2067.59</v>
+        <v>2238.79</v>
       </c>
       <c r="N6" s="11" t="n">
-        <v>2338.89</v>
+        <v>2510.09</v>
       </c>
       <c r="O6" s="11" t="n">
-        <v>2336.69</v>
+        <v>2507.89</v>
       </c>
       <c r="P6" s="11" t="n">
-        <v>2334.09</v>
+        <v>2505.29</v>
       </c>
       <c r="Q6" s="11" t="n">
-        <v>2332.19</v>
+        <v>2503.39</v>
       </c>
       <c r="R6" s="11" t="n">
-        <v>2330.49</v>
+        <v>2501.69</v>
       </c>
       <c r="S6" s="11" t="n">
-        <v>2330.49</v>
+        <v>2501.69</v>
       </c>
       <c r="T6" s="10" t="inlineStr">
         <is>
@@ -924,34 +924,34 @@
         <v>27.84</v>
       </c>
       <c r="J7" s="14" t="n">
-        <v>143.6</v>
+        <v>229.2</v>
       </c>
       <c r="K7" s="14" t="n">
-        <v>273.39</v>
+        <v>358.99</v>
       </c>
       <c r="L7" s="14" t="n">
-        <v>377.79</v>
+        <v>548.99</v>
       </c>
       <c r="M7" s="14" t="n">
-        <v>377.79</v>
+        <v>548.99</v>
       </c>
       <c r="N7" s="14" t="n">
-        <v>377.79</v>
+        <v>548.99</v>
       </c>
       <c r="O7" s="14" t="n">
-        <v>375.59</v>
+        <v>546.79</v>
       </c>
       <c r="P7" s="14" t="n">
-        <v>372.99</v>
+        <v>544.1900000000001</v>
       </c>
       <c r="Q7" s="14" t="n">
-        <v>371.09</v>
+        <v>542.29</v>
       </c>
       <c r="R7" s="14" t="n">
-        <v>369.39</v>
+        <v>540.59</v>
       </c>
       <c r="S7" s="14" t="n">
-        <v>369.39</v>
+        <v>540.59</v>
       </c>
       <c r="T7" s="13" t="inlineStr">
         <is>
@@ -1040,34 +1040,34 @@
         <v>15.21</v>
       </c>
       <c r="J9" s="17" t="n">
-        <v>155.47</v>
+        <v>241.07</v>
       </c>
       <c r="K9" s="17" t="n">
-        <v>233.81</v>
+        <v>319.41</v>
       </c>
       <c r="L9" s="17" t="n">
-        <v>338.21</v>
+        <v>509.41</v>
       </c>
       <c r="M9" s="17" t="n">
-        <v>338.21</v>
+        <v>509.41</v>
       </c>
       <c r="N9" s="17" t="n">
-        <v>338.21</v>
+        <v>509.41</v>
       </c>
       <c r="O9" s="17" t="n">
-        <v>338.21</v>
+        <v>509.41</v>
       </c>
       <c r="P9" s="17" t="n">
-        <v>338.21</v>
+        <v>509.41</v>
       </c>
       <c r="Q9" s="17" t="n">
-        <v>338.21</v>
+        <v>509.41</v>
       </c>
       <c r="R9" s="17" t="n">
-        <v>338.21</v>
+        <v>509.41</v>
       </c>
       <c r="S9" s="17" t="n">
-        <v>335.87</v>
+        <v>507.07</v>
       </c>
       <c r="T9" s="16" t="inlineStr">
         <is>
@@ -1115,34 +1115,34 @@
         <v>1993.36</v>
       </c>
       <c r="J10" s="20" t="n">
-        <v>2111.89</v>
+        <v>2197.49</v>
       </c>
       <c r="K10" s="20" t="n">
-        <v>2360.51</v>
+        <v>2446.11</v>
       </c>
       <c r="L10" s="20" t="n">
-        <v>2465.37</v>
+        <v>2636.57</v>
       </c>
       <c r="M10" s="20" t="n">
-        <v>2465.57</v>
+        <v>2636.77</v>
       </c>
       <c r="N10" s="20" t="n">
-        <v>2465.77</v>
+        <v>2636.97</v>
       </c>
       <c r="O10" s="20" t="n">
-        <v>2463.77</v>
+        <v>2634.97</v>
       </c>
       <c r="P10" s="20" t="n">
-        <v>2461.37</v>
+        <v>2632.57</v>
       </c>
       <c r="Q10" s="20" t="n">
-        <v>2459.62</v>
+        <v>2630.82</v>
       </c>
       <c r="R10" s="20" t="n">
-        <v>2458.07</v>
+        <v>2629.27</v>
       </c>
       <c r="S10" s="20" t="n">
-        <v>544.86</v>
+        <v>716.0599999999999</v>
       </c>
       <c r="T10" s="19" t="inlineStr">
         <is>
@@ -1190,34 +1190,34 @@
         <v>1993.36</v>
       </c>
       <c r="J11" s="20" t="n">
-        <v>3129.73</v>
+        <v>3215.33</v>
       </c>
       <c r="K11" s="20" t="n">
-        <v>4050.31</v>
+        <v>4135.91</v>
       </c>
       <c r="L11" s="20" t="n">
-        <v>4155.17</v>
+        <v>4326.37</v>
       </c>
       <c r="M11" s="20" t="n">
-        <v>4155.37</v>
+        <v>4326.57</v>
       </c>
       <c r="N11" s="20" t="n">
-        <v>4426.87</v>
+        <v>4598.07</v>
       </c>
       <c r="O11" s="20" t="n">
-        <v>4424.87</v>
+        <v>4596.07</v>
       </c>
       <c r="P11" s="20" t="n">
-        <v>4422.47</v>
+        <v>4593.67</v>
       </c>
       <c r="Q11" s="20" t="n">
-        <v>4420.72</v>
+        <v>4591.92</v>
       </c>
       <c r="R11" s="20" t="n">
-        <v>4419.17</v>
+        <v>4590.37</v>
       </c>
       <c r="S11" s="20" t="n">
-        <v>2505.96</v>
+        <v>2677.16</v>
       </c>
       <c r="T11" s="19" t="inlineStr">
         <is>
@@ -1306,34 +1306,34 @@
         <v>27.84</v>
       </c>
       <c r="J13" s="11" t="n">
-        <v>1161.44</v>
+        <v>1247.04</v>
       </c>
       <c r="K13" s="11" t="n">
-        <v>1963.19</v>
+        <v>2048.79</v>
       </c>
       <c r="L13" s="11" t="n">
-        <v>2067.59</v>
+        <v>2238.79</v>
       </c>
       <c r="M13" s="11" t="n">
-        <v>2067.59</v>
+        <v>2238.79</v>
       </c>
       <c r="N13" s="11" t="n">
-        <v>2338.89</v>
+        <v>2510.09</v>
       </c>
       <c r="O13" s="11" t="n">
-        <v>2336.69</v>
+        <v>2507.89</v>
       </c>
       <c r="P13" s="11" t="n">
-        <v>2334.09</v>
+        <v>2505.29</v>
       </c>
       <c r="Q13" s="11" t="n">
-        <v>2332.19</v>
+        <v>2503.39</v>
       </c>
       <c r="R13" s="11" t="n">
-        <v>2330.49</v>
+        <v>2501.69</v>
       </c>
       <c r="S13" s="11" t="n">
-        <v>2330.49</v>
+        <v>2501.69</v>
       </c>
       <c r="T13" s="10" t="inlineStr">
         <is>
@@ -1364,34 +1364,34 @@
         <v>27.84</v>
       </c>
       <c r="J14" s="14" t="n">
-        <v>143.6</v>
+        <v>229.2</v>
       </c>
       <c r="K14" s="14" t="n">
-        <v>273.39</v>
+        <v>358.99</v>
       </c>
       <c r="L14" s="14" t="n">
-        <v>377.79</v>
+        <v>548.99</v>
       </c>
       <c r="M14" s="14" t="n">
-        <v>377.79</v>
+        <v>548.99</v>
       </c>
       <c r="N14" s="14" t="n">
-        <v>377.79</v>
+        <v>548.99</v>
       </c>
       <c r="O14" s="14" t="n">
-        <v>375.59</v>
+        <v>546.79</v>
       </c>
       <c r="P14" s="14" t="n">
-        <v>372.99</v>
+        <v>544.1900000000001</v>
       </c>
       <c r="Q14" s="14" t="n">
-        <v>371.09</v>
+        <v>542.29</v>
       </c>
       <c r="R14" s="14" t="n">
-        <v>369.39</v>
+        <v>540.59</v>
       </c>
       <c r="S14" s="14" t="n">
-        <v>369.39</v>
+        <v>540.59</v>
       </c>
       <c r="T14" s="13" t="inlineStr">
         <is>
@@ -1480,34 +1480,34 @@
         <v>15.21</v>
       </c>
       <c r="J16" s="17" t="n">
-        <v>155.47</v>
+        <v>241.07</v>
       </c>
       <c r="K16" s="17" t="n">
-        <v>233.81</v>
+        <v>319.41</v>
       </c>
       <c r="L16" s="17" t="n">
-        <v>338.21</v>
+        <v>509.41</v>
       </c>
       <c r="M16" s="17" t="n">
-        <v>338.21</v>
+        <v>509.41</v>
       </c>
       <c r="N16" s="17" t="n">
-        <v>338.21</v>
+        <v>509.41</v>
       </c>
       <c r="O16" s="17" t="n">
-        <v>338.21</v>
+        <v>509.41</v>
       </c>
       <c r="P16" s="17" t="n">
-        <v>338.21</v>
+        <v>509.41</v>
       </c>
       <c r="Q16" s="17" t="n">
-        <v>338.21</v>
+        <v>509.41</v>
       </c>
       <c r="R16" s="17" t="n">
-        <v>338.21</v>
+        <v>509.41</v>
       </c>
       <c r="S16" s="17" t="n">
-        <v>335.87</v>
+        <v>507.07</v>
       </c>
       <c r="T16" s="16" t="inlineStr">
         <is>
@@ -1555,34 +1555,34 @@
         <v>1993.36</v>
       </c>
       <c r="J17" s="20" t="n">
-        <v>2111.89</v>
+        <v>2197.49</v>
       </c>
       <c r="K17" s="20" t="n">
-        <v>2360.51</v>
+        <v>2446.11</v>
       </c>
       <c r="L17" s="20" t="n">
-        <v>2465.37</v>
+        <v>2636.57</v>
       </c>
       <c r="M17" s="20" t="n">
-        <v>2465.57</v>
+        <v>2636.77</v>
       </c>
       <c r="N17" s="20" t="n">
-        <v>2465.77</v>
+        <v>2636.97</v>
       </c>
       <c r="O17" s="20" t="n">
-        <v>2463.77</v>
+        <v>2634.97</v>
       </c>
       <c r="P17" s="20" t="n">
-        <v>2461.37</v>
+        <v>2632.57</v>
       </c>
       <c r="Q17" s="20" t="n">
-        <v>2459.62</v>
+        <v>2630.82</v>
       </c>
       <c r="R17" s="20" t="n">
-        <v>2458.07</v>
+        <v>2629.27</v>
       </c>
       <c r="S17" s="20" t="n">
-        <v>544.86</v>
+        <v>716.0599999999999</v>
       </c>
       <c r="T17" s="19" t="inlineStr">
         <is>
@@ -1630,34 +1630,34 @@
         <v>1993.36</v>
       </c>
       <c r="J18" s="20" t="n">
-        <v>3129.73</v>
+        <v>3215.33</v>
       </c>
       <c r="K18" s="20" t="n">
-        <v>4050.31</v>
+        <v>4135.91</v>
       </c>
       <c r="L18" s="20" t="n">
-        <v>4155.17</v>
+        <v>4326.37</v>
       </c>
       <c r="M18" s="20" t="n">
-        <v>4155.37</v>
+        <v>4326.57</v>
       </c>
       <c r="N18" s="20" t="n">
-        <v>4426.87</v>
+        <v>4598.07</v>
       </c>
       <c r="O18" s="20" t="n">
-        <v>4424.87</v>
+        <v>4596.07</v>
       </c>
       <c r="P18" s="20" t="n">
-        <v>4422.47</v>
+        <v>4593.67</v>
       </c>
       <c r="Q18" s="20" t="n">
-        <v>4420.72</v>
+        <v>4591.92</v>
       </c>
       <c r="R18" s="20" t="n">
-        <v>4419.17</v>
+        <v>4590.37</v>
       </c>
       <c r="S18" s="20" t="n">
-        <v>2505.96</v>
+        <v>2677.16</v>
       </c>
       <c r="T18" s="19" t="inlineStr">
         <is>
@@ -1942,68 +1942,54 @@
     <row r="23">
       <c r="A23" s="24" t="inlineStr">
         <is>
-          <t>ФГБУ "ЦЖКУ"  Минобороны России ( котельные №97 в/г 135)</t>
-        </is>
-      </c>
-      <c r="B23" s="25" t="inlineStr">
-        <is>
-          <t>Минобороны</t>
-        </is>
-      </c>
-      <c r="C23" s="25" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="D23" s="25" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="E23" s="25" t="n">
-        <v>18</v>
-      </c>
+          <t>Действующие потребители</t>
+        </is>
+      </c>
+      <c r="B23" s="25" t="inlineStr"/>
+      <c r="C23" s="25" t="inlineStr"/>
+      <c r="D23" s="25" t="inlineStr"/>
+      <c r="E23" s="25" t="inlineStr"/>
       <c r="F23" s="26" t="n">
-        <v>0.8100000000000001</v>
+        <v>715.65</v>
       </c>
       <c r="G23" s="26" t="n">
-        <v>0.68</v>
+        <v>734.4400000000001</v>
       </c>
       <c r="H23" s="26" t="n">
-        <v>0.8200000000000001</v>
+        <v>757.45</v>
       </c>
       <c r="I23" s="26" t="n">
-        <v>0.8200000000000001</v>
+        <v>771.14</v>
       </c>
       <c r="J23" s="26" t="n">
-        <v>0.8200000000000001</v>
+        <v>771.41</v>
       </c>
       <c r="K23" s="26" t="n">
-        <v>0.8200000000000001</v>
+        <v>781.03</v>
       </c>
       <c r="L23" s="26" t="n">
-        <v>0.8200000000000001</v>
+        <v>781.49</v>
       </c>
       <c r="M23" s="26" t="n">
-        <v>0.8200000000000001</v>
+        <v>781.6900000000001</v>
       </c>
       <c r="N23" s="26" t="n">
-        <v>0.8200000000000001</v>
+        <v>781.89</v>
       </c>
       <c r="O23" s="26" t="n">
-        <v>0.8200000000000001</v>
+        <v>782.09</v>
       </c>
       <c r="P23" s="26" t="n">
-        <v>0.8200000000000001</v>
+        <v>782.29</v>
       </c>
       <c r="Q23" s="26" t="n">
-        <v>0.8200000000000001</v>
+        <v>782.4400000000001</v>
       </c>
       <c r="R23" s="26" t="n">
-        <v>0.8200000000000001</v>
+        <v>782.59</v>
       </c>
       <c r="S23" s="26" t="n">
-        <v>0.01</v>
+        <v>66.94</v>
       </c>
       <c r="T23" s="25" t="inlineStr">
         <is>
@@ -2014,7 +2000,7 @@
     <row r="24">
       <c r="A24" s="24" t="inlineStr">
         <is>
-          <t>Действующие потребители</t>
+          <t>Прочие потребители</t>
         </is>
       </c>
       <c r="B24" s="25" t="inlineStr"/>
@@ -2022,46 +2008,46 @@
       <c r="D24" s="25" t="inlineStr"/>
       <c r="E24" s="25" t="inlineStr"/>
       <c r="F24" s="26" t="n">
-        <v>747.16</v>
+        <v>32.32</v>
       </c>
       <c r="G24" s="26" t="n">
-        <v>748.17</v>
+        <v>14.41</v>
       </c>
       <c r="H24" s="26" t="n">
-        <v>774.15</v>
+        <v>17.52</v>
       </c>
       <c r="I24" s="26" t="n">
-        <v>787.84</v>
+        <v>17.52</v>
       </c>
       <c r="J24" s="26" t="n">
-        <v>790.61</v>
+        <v>20.02</v>
       </c>
       <c r="K24" s="26" t="n">
-        <v>800.38</v>
+        <v>20.17</v>
       </c>
       <c r="L24" s="26" t="n">
-        <v>800.84</v>
+        <v>20.17</v>
       </c>
       <c r="M24" s="26" t="n">
-        <v>801.04</v>
+        <v>20.17</v>
       </c>
       <c r="N24" s="26" t="n">
-        <v>801.24</v>
+        <v>20.17</v>
       </c>
       <c r="O24" s="26" t="n">
-        <v>801.4400000000001</v>
+        <v>20.17</v>
       </c>
       <c r="P24" s="26" t="n">
-        <v>801.64</v>
+        <v>20.17</v>
       </c>
       <c r="Q24" s="26" t="n">
-        <v>801.79</v>
+        <v>20.17</v>
       </c>
       <c r="R24" s="26" t="n">
-        <v>801.9400000000001</v>
+        <v>20.17</v>
       </c>
       <c r="S24" s="26" t="n">
-        <v>54.78</v>
+        <v>-12.15</v>
       </c>
       <c r="T24" s="25" t="inlineStr">
         <is>
@@ -2092,34 +2078,34 @@
         <v>27.84</v>
       </c>
       <c r="J25" s="23" t="n">
-        <v>143.6</v>
+        <v>229.2</v>
       </c>
       <c r="K25" s="23" t="n">
-        <v>273.39</v>
+        <v>358.99</v>
       </c>
       <c r="L25" s="23" t="n">
-        <v>377.79</v>
+        <v>548.99</v>
       </c>
       <c r="M25" s="23" t="n">
-        <v>377.79</v>
+        <v>548.99</v>
       </c>
       <c r="N25" s="23" t="n">
-        <v>377.79</v>
+        <v>548.99</v>
       </c>
       <c r="O25" s="23" t="n">
-        <v>375.59</v>
+        <v>546.79</v>
       </c>
       <c r="P25" s="23" t="n">
-        <v>372.99</v>
+        <v>544.1900000000001</v>
       </c>
       <c r="Q25" s="23" t="n">
-        <v>371.09</v>
+        <v>542.29</v>
       </c>
       <c r="R25" s="23" t="n">
-        <v>369.39</v>
+        <v>540.59</v>
       </c>
       <c r="S25" s="23" t="n">
-        <v>369.39</v>
+        <v>540.59</v>
       </c>
       <c r="T25" s="22" t="inlineStr">
         <is>
@@ -2418,68 +2404,68 @@
     <row r="30">
       <c r="A30" s="24" t="inlineStr">
         <is>
-          <t>АО "Каспийский трубопроводный консорциум - Р"(НПС-4А)</t>
+          <t>ГТУ ТЭЦ (объект инфраструктурного инвестора)</t>
         </is>
       </c>
       <c r="B30" s="25" t="inlineStr">
         <is>
-          <t>Нефтяная</t>
+          <t>Электроэнергетика</t>
         </is>
       </c>
       <c r="C30" s="25" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="D30" s="25" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="E30" s="25" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="F30" s="26" t="n">
         <v>0</v>
       </c>
       <c r="G30" s="26" t="n">
-        <v>1.68</v>
+        <v>0</v>
       </c>
       <c r="H30" s="26" t="n">
-        <v>1.68</v>
+        <v>0</v>
       </c>
       <c r="I30" s="26" t="n">
-        <v>12.59</v>
+        <v>0</v>
       </c>
       <c r="J30" s="26" t="n">
-        <v>12.59</v>
+        <v>85.59999999999999</v>
       </c>
       <c r="K30" s="26" t="n">
-        <v>14</v>
+        <v>85.59999999999999</v>
       </c>
       <c r="L30" s="26" t="n">
-        <v>14</v>
+        <v>171.2</v>
       </c>
       <c r="M30" s="26" t="n">
-        <v>14</v>
+        <v>171.2</v>
       </c>
       <c r="N30" s="26" t="n">
-        <v>14</v>
+        <v>171.2</v>
       </c>
       <c r="O30" s="26" t="n">
-        <v>11.8</v>
+        <v>171.2</v>
       </c>
       <c r="P30" s="26" t="n">
-        <v>9.199999999999999</v>
+        <v>171.2</v>
       </c>
       <c r="Q30" s="26" t="n">
-        <v>7.3</v>
+        <v>171.2</v>
       </c>
       <c r="R30" s="26" t="n">
-        <v>5.6</v>
+        <v>171.2</v>
       </c>
       <c r="S30" s="26" t="n">
-        <v>5.6</v>
+        <v>171.2</v>
       </c>
       <c r="T30" s="25" t="inlineStr">
         <is>
@@ -2501,43 +2487,43 @@
         <v>0</v>
       </c>
       <c r="G31" s="26" t="n">
-        <v>0.32</v>
+        <v>2</v>
       </c>
       <c r="H31" s="26" t="n">
-        <v>6</v>
+        <v>7.68</v>
       </c>
       <c r="I31" s="26" t="n">
-        <v>15.25</v>
+        <v>27.84</v>
       </c>
       <c r="J31" s="26" t="n">
-        <v>24.61</v>
+        <v>37.2</v>
       </c>
       <c r="K31" s="26" t="n">
-        <v>52.59</v>
+        <v>66.59</v>
       </c>
       <c r="L31" s="26" t="n">
-        <v>62.39</v>
+        <v>76.39</v>
       </c>
       <c r="M31" s="26" t="n">
-        <v>62.39</v>
+        <v>76.39</v>
       </c>
       <c r="N31" s="26" t="n">
-        <v>62.39</v>
+        <v>76.39</v>
       </c>
       <c r="O31" s="26" t="n">
-        <v>62.39</v>
+        <v>74.19</v>
       </c>
       <c r="P31" s="26" t="n">
-        <v>62.39</v>
+        <v>71.59</v>
       </c>
       <c r="Q31" s="26" t="n">
-        <v>62.39</v>
+        <v>69.69</v>
       </c>
       <c r="R31" s="26" t="n">
-        <v>62.39</v>
+        <v>67.98999999999999</v>
       </c>
       <c r="S31" s="26" t="n">
-        <v>62.39</v>
+        <v>67.98999999999999</v>
       </c>
       <c r="T31" s="25" t="inlineStr">
         <is>

</xml_diff>